<commit_message>
final deployment under test
</commit_message>
<xml_diff>
--- a/results_report.xlsx
+++ b/results_report.xlsx
@@ -576,6 +576,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -601,6 +604,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -626,6 +632,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -651,6 +660,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -670,6 +682,834 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId46"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId47"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId48"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId49"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -972,7 +1812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1314,6 +2154,138 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="105" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>005663</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:27:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="105" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>005663</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:31:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="105" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>005663</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-05-25 15:02:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="105" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>005663</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-06-01 10:04:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="105" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>005663</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-06-01 10:24:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="105" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>005663</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-06-01 10:30:44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
third trial for devops concept
</commit_message>
<xml_diff>
--- a/results_report.xlsx
+++ b/results_report.xlsx
@@ -436,6 +436,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -461,6 +464,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -480,6 +486,84 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="1285875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -782,7 +866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -919,6 +1003,28 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="105" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2511TL005663ISI</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>005663</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:40:18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>